<commit_message>
BOM Format set for all design BOMs.
</commit_message>
<xml_diff>
--- a/Design Files/Test Power Module PCB Design-v1.0.0/BOM/Test Power Module PCB Design v1.0.0.xlsx
+++ b/Design Files/Test Power Module PCB Design-v1.0.0/BOM/Test Power Module PCB Design v1.0.0.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20410"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\gerholdvoorde-dronebms\Design Files\Test Power Module PCB Design v1.0.0\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\gerholdvoorde-dronebms\Design Files\Test Power Module PCB Design-v1.0.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5AC938-4F5F-4E1A-ABC8-D84D93E02CAC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
   <si>
     <t>#</t>
   </si>
@@ -112,9 +111,6 @@
     <t>RT0603BRD0710KL</t>
   </si>
   <si>
-    <t>MANUFACTURER</t>
-  </si>
-  <si>
     <t>BOOMELE</t>
   </si>
   <si>
@@ -149,12 +145,18 @@
   </si>
   <si>
     <t>Custom</t>
+  </si>
+  <si>
+    <t>Manufacturer</t>
+  </si>
+  <si>
+    <t>RC0603FR-0730KL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -639,7 +641,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -690,16 +692,16 @@
         <v>26</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -724,10 +726,10 @@
         <v>27</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -750,16 +752,16 @@
         <v>16</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G4" s="10" t="s">
         <v>28</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J4" s="9">
         <v>4</v>
@@ -782,16 +784,16 @@
         <v>17</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>23</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J5" s="7">
         <v>5</v>
@@ -804,7 +806,9 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="13"/>
+      <c r="C6" s="12" t="s">
+        <v>5</v>
+      </c>
       <c r="D6" s="9" t="s">
         <v>11</v>
       </c>
@@ -814,10 +818,14 @@
       <c r="F6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="9"/>
+      <c r="G6" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>33</v>
+      </c>
       <c r="I6" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -846,10 +854,10 @@
         <v>29</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -872,16 +880,16 @@
         <v>20</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G8" s="10" t="s">
         <v>25</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>

</xml_diff>